<commit_message>
Day 26: Supplier risk variation and monthly financial loss tracking
</commit_message>
<xml_diff>
--- a/static/exports/wastage_risk_report.xlsx
+++ b/static/exports/wastage_risk_report.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,12 +451,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cefixime 200mg Capsules</t>
+          <t>Amoxicillin 250mg</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CEF-2026-18</t>
+          <t>B2026-102</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -468,7 +468,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -479,12 +479,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Amoxicillin 250mg</t>
+          <t>Cefixime 200mg Capsules</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>B2026-102</t>
+          <t>CEF-2026-18</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -507,16 +507,16 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>IV Saline 500ml</t>
+          <t>Cardiac Stent Implant</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IV-2026-77</t>
+          <t>IMP-2026-44</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-33</v>
+        <v>-26</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -524,7 +524,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -576,31 +576,31 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Prioritize using this batch soon</t>
+          <t>Transfer to another department or return to supplier</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Azithromycin 500mg</t>
+          <t>Paracetamol 500mg</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AZI-2026-21</t>
+          <t>B2026-101</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>44</v>
+        <v>-15</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -619,72 +619,72 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Paracetamol 500mg</t>
+          <t>dolo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>B2026-101</t>
+          <t>123</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-15</v>
+        <v>270</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Prioritize using this batch soon</t>
+          <t>Use first per normal FEFO order</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Cardiac Stent Implant</t>
+          <t>Azithromycin 500mg</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>IMP-2026-44</t>
+          <t>AZI-2026-21</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-26</v>
+        <v>44</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Prioritize using this batch soon</t>
+          <t>Use first per normal FEFO order</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>dolo</t>
+          <t>N95 Respirator Masks (Box of 50)</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>123</t>
+          <t>N95-2026-07</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>270</v>
+        <v>140</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -703,16 +703,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Insulin Vials</t>
+          <t>Suture Kit (Absorbable)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>INS-2026-14</t>
+          <t>SUT-2026-09</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>164</v>
+        <v>55</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -731,16 +731,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Suture Kit (Absorbable)</t>
+          <t>Insulin Vials</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>SUT-2026-09</t>
+          <t>INS-2026-14</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>55</v>
+        <v>164</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -759,16 +759,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Surgical Gloves (Box)</t>
+          <t>Knee Replacement Implant</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>SG-2026-05</t>
+          <t>IMP-2026-19</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>55</v>
+        <v>235</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -776,7 +776,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -787,16 +787,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>N95 Respirator Masks (Box of 50)</t>
+          <t>Surgical Gloves (Box)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>N95-2026-07</t>
+          <t>SG-2026-05</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>140</v>
+        <v>55</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -815,16 +815,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Knee Replacement Implant</t>
+          <t>Orthopedic Implant Kit</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>IMP-2026-19</t>
+          <t>IMP-2026-09</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>235</v>
+        <v>100</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -832,37 +832,9 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F15" t="inlineStr">
-        <is>
-          <t>Use first per normal FEFO order</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Orthopedic Implant Kit</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>IMP-2026-09</t>
-        </is>
-      </c>
-      <c r="C16" t="n">
-        <v>100</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="inlineStr">
         <is>
           <t>Use first per normal FEFO order</t>
         </is>

</xml_diff>